<commit_message>
Add role-based auth flow for dashboard and seed users
</commit_message>
<xml_diff>
--- a/templates/meta_ads_report_template.xlsx
+++ b/templates/meta_ads_report_template.xlsx
@@ -12,6 +12,7 @@
     <sheet name="telegram_targets" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="run_logs" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="manual_run_queue" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="app_users" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -659,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -715,30 +716,30 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>META_ADSET_BREAKDOWN</t>
+          <t>META_FULL_METRICS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>MIN_SPEND</t>
+          <t>CTR_LOW</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>10000</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Minimum spend to show adset</t>
+          <t>Low CTR threshold</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>META_ADSET_PERFORMANCE</t>
+          <t>META_ADSET_BREAKDOWN</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -754,7 +755,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Minimum spend to evaluate funnel</t>
+          <t>Minimum spend to show adset</t>
         </is>
       </c>
     </row>
@@ -766,41 +767,41 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CPR_HIGH</t>
+          <t>MIN_SPEND</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>70000</v>
+        <v>10000</v>
       </c>
       <c r="D5" t="n">
         <v>1</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>High CPR threshold</t>
+          <t>Minimum spend to evaluate funnel</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>META_TOP_ADS_PROFIT</t>
+          <t>META_ADSET_PERFORMANCE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MIN_SPEND</t>
+          <t>CPR_HIGH</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10000</v>
+        <v>70000</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Minimum spend for top ads</t>
+          <t>High CPR threshold</t>
         </is>
       </c>
     </row>
@@ -812,41 +813,41 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TOP_LIMIT</t>
+          <t>MIN_SPEND</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>10</v>
+        <v>10000</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Max rows in ranking</t>
+          <t>Minimum spend for top ads</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>META_TOP_ADS_WINNER</t>
+          <t>META_TOP_ADS_PROFIT</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>WINNER_MIN_SPEND</t>
+          <t>TOP_LIMIT</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>30000</v>
+        <v>10</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Minimum spend for winner</t>
+          <t>Max rows in ranking</t>
         </is>
       </c>
     </row>
@@ -858,18 +859,18 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>WINNER_MIN_ROAS</t>
+          <t>MIN_SPEND</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>10000</v>
       </c>
       <c r="D9" t="n">
         <v>1</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Minimum ROAS for winner</t>
+          <t>Minimum spend for candidates</t>
         </is>
       </c>
     </row>
@@ -881,18 +882,18 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>WINNER_MIN_BUY</t>
+          <t>WINNER_MIN_SPEND</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>30000</v>
       </c>
       <c r="D10" t="n">
         <v>1</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Minimum purchase for winner</t>
+          <t>Minimum spend for winner</t>
         </is>
       </c>
     </row>
@@ -904,64 +905,64 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>TOP_LIMIT</t>
+          <t>WINNER_MIN_ROAS</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Max winner rows</t>
+          <t>Minimum ROAS for winner</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>META_FUNNEL_ALERT</t>
+          <t>META_TOP_ADS_WINNER</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MIN_SPEND</t>
+          <t>WINNER_MIN_BUY</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>10000</v>
+        <v>2</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Minimum spend for alert check</t>
+          <t>Minimum purchase for winner</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>META_FUNNEL_ALERT</t>
+          <t>META_TOP_ADS_WINNER</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CPM_SPIKE</t>
+          <t>TOP_LIMIT</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>100000</v>
+        <v>10</v>
       </c>
       <c r="D13" t="n">
         <v>1</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CPM spike threshold</t>
+          <t>Max winner rows</t>
         </is>
       </c>
     </row>
@@ -973,64 +974,64 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CTR_LOW</t>
+          <t>MIN_SPEND</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>10000</v>
       </c>
       <c r="D14" t="n">
         <v>1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Low CTR threshold</t>
+          <t>Minimum spend for alert check</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>META_CREATIVE_FATIGUE</t>
+          <t>META_FUNNEL_ALERT</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>FATIGUE_MIN_SPEND</t>
+          <t>CPM_SPIKE</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="D15" t="n">
         <v>1</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Minimum spend for fatigue check</t>
+          <t>CPM spike threshold</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>META_CREATIVE_FATIGUE</t>
+          <t>META_FUNNEL_ALERT</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>FATIGUE_CTR_MAX</t>
+          <t>CTR_LOW</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.8</v>
+        <v>2</v>
       </c>
       <c r="D16" t="n">
         <v>1</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Max CTR before fatigue</t>
+          <t>Low CTR threshold</t>
         </is>
       </c>
     </row>
@@ -1042,18 +1043,18 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>FATIGUE_CPM_MIN</t>
+          <t>SPEND_NO_PURCHASE</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="D17" t="n">
         <v>1</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Min CPM before fatigue</t>
+          <t>Pause no purchase threshold</t>
         </is>
       </c>
     </row>
@@ -1065,18 +1066,156 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>FATIGUE_MIN_SPEND</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>30000</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Minimum spend for fatigue check</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>META_CREATIVE_FATIGUE</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>FATIGUE_CTR_MAX</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Max CTR before fatigue</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>META_CREATIVE_FATIGUE</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>FATIGUE_CPM_MIN</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Min CPM before fatigue</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>META_CREATIVE_FATIGUE</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>SCALE_ROAS_MIN</t>
         </is>
       </c>
-      <c r="C18" t="n">
+      <c r="C21" t="n">
         <v>1.5</v>
       </c>
-      <c r="D18" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" t="inlineStr">
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>ROAS minimum for scale suggestion</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>META_CREATIVE_FATIGUE</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SCALE_CTR_MIN</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>CTR min for scale</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>META_CREATIVE_FATIGUE</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>PAUSE_ROAS_MAX</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ROAS max for pause</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>META_CREATIVE_FATIGUE</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>CPM_SPIKE</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>100000</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>CPM spike threshold</t>
         </is>
       </c>
     </row>
@@ -1291,4 +1430,70 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>user_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>password_hash</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>password_salt</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>is_active</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>last_login_at</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>